<commit_message>
Compare Mtion Mini Doppler and non-Doppler using Mark's data
</commit_message>
<xml_diff>
--- a/sessions/contacts/mark/analysis/doppler_vs_positional.xlsx
+++ b/sessions/contacts/mark/analysis/doppler_vs_positional.xlsx
@@ -8,12 +8,13 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl$\Ubuntu\home\mike\projects\docs\gps-guides\sessions\contacts\mark\analysis\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FCAA3399-1EFD-41A7-A71B-6314BCF5DA01}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{67E8976D-B926-43E7-90D7-7B1CBAD358B9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{1A0D1499-61F0-4420-A350-725B2B0FF3B8}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" activeTab="1" xr2:uid="{1A0D1499-61F0-4420-A350-725B2B0FF3B8}"/>
   </bookViews>
   <sheets>
     <sheet name="fenix-5" sheetId="1" r:id="rId1"/>
+    <sheet name="motion-mini" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="181029"/>
   <extLst>
@@ -33,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11" uniqueCount="9">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="12">
   <si>
     <t>doppler</t>
   </si>
@@ -60,6 +61,15 @@
   </si>
   <si>
     <t>diff</t>
+  </si>
+  <si>
+    <t>+/-</t>
+  </si>
+  <si>
+    <t>Note: 4 runs could not be matched up for some reason!</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Note time difference of 2 seconds </t>
   </si>
 </sst>
 </file>
@@ -103,11 +113,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="21" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -410,6 +421,472 @@
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
               <c16:uniqueId val="{00000001-AC77-4052-B24A-4D93046CB5B9}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:dLbls>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+        </c:dLbls>
+        <c:gapWidth val="150"/>
+        <c:axId val="567313464"/>
+        <c:axId val="567318712"/>
+      </c:barChart>
+      <c:catAx>
+        <c:axId val="567313464"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="b"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:solidFill>
+              <a:schemeClr val="tx1">
+                <a:lumMod val="15000"/>
+                <a:lumOff val="85000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="567318712"/>
+        <c:crosses val="autoZero"/>
+        <c:auto val="1"/>
+        <c:lblAlgn val="ctr"/>
+        <c:lblOffset val="100"/>
+        <c:noMultiLvlLbl val="0"/>
+      </c:catAx>
+      <c:valAx>
+        <c:axId val="567318712"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+          <c:min val="0"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="l"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="15000"/>
+                  <a:lumOff val="85000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln>
+            <a:noFill/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="567313464"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="between"/>
+      </c:valAx>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+    </c:plotArea>
+    <c:legend>
+      <c:legendPos val="t"/>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="en-US"/>
+        </a:p>
+      </c:txPr>
+    </c:legend>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
+    <c:extLst>
+      <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
+        <c16r3:dataDisplayOptions16>
+          <c16r3:dispNaAsBlank val="1"/>
+        </c16r3:dataDisplayOptions16>
+      </c:ext>
+    </c:extLst>
+    <c:showDLblsOverMax val="0"/>
+  </c:chart>
+  <c:spPr>
+    <a:solidFill>
+      <a:schemeClr val="bg1"/>
+    </a:solidFill>
+    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+      <a:solidFill>
+        <a:schemeClr val="tx1">
+          <a:lumMod val="15000"/>
+          <a:lumOff val="85000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:round/>
+    </a:ln>
+    <a:effectLst/>
+  </c:spPr>
+  <c:txPr>
+    <a:bodyPr/>
+    <a:lstStyle/>
+    <a:p>
+      <a:pPr>
+        <a:defRPr/>
+      </a:pPr>
+      <a:endParaRPr lang="en-US"/>
+    </a:p>
+  </c:txPr>
+  <c:printSettings>
+    <c:headerFooter/>
+    <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
+    <c:pageSetup/>
+  </c:printSettings>
+</c:chartSpace>
+</file>
+
+<file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+  <c:date1904 val="0"/>
+  <c:lang val="en-US"/>
+  <c:roundedCorners val="0"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
+      <c14:style val="102"/>
+    </mc:Choice>
+    <mc:Fallback>
+      <c:style val="2"/>
+    </mc:Fallback>
+  </mc:AlternateContent>
+  <c:chart>
+    <c:title>
+      <c:tx>
+        <c:rich>
+          <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:r>
+              <a:rPr lang="en-GB"/>
+              <a:t>Motion Mini</a:t>
+            </a:r>
+          </a:p>
+          <a:p>
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:rPr lang="en-GB" sz="1200"/>
+              <a:t>Twenty 250m runs - Doppler</a:t>
+            </a:r>
+            <a:r>
+              <a:rPr lang="en-GB" sz="1200" baseline="0"/>
+              <a:t> vs Non-Doppler</a:t>
+            </a:r>
+            <a:endParaRPr lang="en-GB" sz="1200"/>
+          </a:p>
+        </c:rich>
+      </c:tx>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="en-US"/>
+        </a:p>
+      </c:txPr>
+    </c:title>
+    <c:autoTitleDeleted val="0"/>
+    <c:plotArea>
+      <c:layout/>
+      <c:barChart>
+        <c:barDir val="col"/>
+        <c:grouping val="clustered"/>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>'motion-mini'!$C$1</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>doppler</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:solidFill>
+              <a:schemeClr val="accent1"/>
+            </a:solidFill>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:invertIfNegative val="0"/>
+          <c:val>
+            <c:numRef>
+              <c:f>'motion-mini'!$C$2:$C$21</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="20"/>
+                <c:pt idx="0">
+                  <c:v>34.914000000000001</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>36.137999999999998</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>29.506</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>35.067999999999998</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>29.300999999999998</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>35.588999999999999</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>28.795999999999999</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>28.797999999999998</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>35.308999999999997</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>35.889000000000003</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>28.018999999999998</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>28.951000000000001</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>35.619999999999997</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>28.478000000000002</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>34.435000000000002</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>33.265000000000001</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000000-27FB-4726-9DB5-7DC59D1D7E3D}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:ser>
+          <c:idx val="1"/>
+          <c:order val="1"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>'motion-mini'!$H$1</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>non-doppler</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:solidFill>
+              <a:schemeClr val="accent2"/>
+            </a:solidFill>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:invertIfNegative val="0"/>
+          <c:val>
+            <c:numRef>
+              <c:f>'motion-mini'!$H$2:$H$21</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="20"/>
+                <c:pt idx="0">
+                  <c:v>34.682000000000002</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>36.226999999999997</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>29.507999999999999</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>34.295000000000002</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>29.334</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>35.558999999999997</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>28.81</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>28.742999999999999</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>35.296999999999997</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>35.857999999999997</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>28.018999999999998</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>28.969000000000001</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>35.479999999999997</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>28.518000000000001</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>34.478999999999999</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>33.347000000000001</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000001-27FB-4726-9DB5-7DC59D1D7E3D}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -655,7 +1132,563 @@
 </cs:colorStyle>
 </file>
 
+<file path=xl/charts/colors2.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
+  <a:schemeClr val="accent1"/>
+  <a:schemeClr val="accent2"/>
+  <a:schemeClr val="accent3"/>
+  <a:schemeClr val="accent4"/>
+  <a:schemeClr val="accent5"/>
+  <a:schemeClr val="accent6"/>
+  <cs:variation/>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+    <a:lumOff val="20000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+    <a:lumOff val="40000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+    <a:lumOff val="30000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+    <a:lumOff val="50000"/>
+  </cs:variation>
+</cs:colorStyle>
+</file>
+
 <file path=xl/charts/style1.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="227">
+  <cs:axisTitle>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:axisTitle>
+  <cs:categoryAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:categoryAxis>
+  <cs:chartArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="bg1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:chartArea>
+  <cs:dataLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="75000"/>
+        <a:lumOff val="25000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataLabel>
+  <cs:dataLabelCallout>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln>
+        <a:solidFill>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+    <cs:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="36576" tIns="18288" rIns="36576" bIns="18288" anchor="ctr" anchorCtr="1">
+      <a:spAutoFit/>
+    </cs:bodyPr>
+  </cs:dataLabelCallout>
+  <cs:dataPoint>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="phClr"/>
+      </a:solidFill>
+    </cs:spPr>
+  </cs:dataPoint>
+  <cs:dataPoint3D>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="phClr"/>
+      </a:solidFill>
+    </cs:spPr>
+  </cs:dataPoint3D>
+  <cs:dataPointLine>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="28575" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointLine>
+  <cs:dataPointMarker>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="phClr"/>
+      </a:solidFill>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointMarker>
+  <cs:dataPointMarkerLayout symbol="circle" size="5"/>
+  <cs:dataPointWireframe>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointWireframe>
+  <cs:dataTable>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataTable>
+  <cs:downBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="dk1">
+          <a:lumMod val="65000"/>
+          <a:lumOff val="35000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:downBar>
+  <cs:dropLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dropLine>
+  <cs:errorBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:errorBar>
+  <cs:floor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:floor>
+  <cs:gridlineMajor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMajor>
+  <cs:gridlineMinor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="5000"/>
+            <a:lumOff val="95000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMinor>
+  <cs:hiLoLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="75000"/>
+            <a:lumOff val="25000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:hiLoLine>
+  <cs:leaderLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:leaderLine>
+  <cs:legend>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:legend>
+  <cs:plotArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea>
+  <cs:plotArea3D mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea3D>
+  <cs:seriesAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:seriesAxis>
+  <cs:seriesLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:seriesLine>
+  <cs:title>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1400" b="0" kern="1200" spc="0" baseline="0"/>
+  </cs:title>
+  <cs:trendline>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:prstDash val="sysDot"/>
+      </a:ln>
+    </cs:spPr>
+  </cs:trendline>
+  <cs:trendlineLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:trendlineLabel>
+  <cs:upBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:upBar>
+  <cs:valueAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:valueAxis>
+  <cs:wall>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:wall>
+</cs:chartStyle>
+</file>
+
+<file path=xl/charts/style2.xml><?xml version="1.0" encoding="utf-8"?>
 <cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="227">
   <cs:axisTitle>
     <cs:lnRef idx="0"/>
@@ -1196,6 +2229,49 @@
           </a:extLst>
         </xdr:cNvPr>
         <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>16</xdr:col>
+      <xdr:colOff>38099</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>180975</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>26</xdr:col>
+      <xdr:colOff>371474</xdr:colOff>
+      <xdr:row>22</xdr:row>
+      <xdr:rowOff>85725</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="2" name="Chart 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{A574F5F7-9181-4080-BF0C-43CF3E499942}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvGraphicFramePr>
+          <a:graphicFrameLocks/>
+        </xdr:cNvGraphicFramePr>
       </xdr:nvGraphicFramePr>
       <xdr:xfrm>
         <a:off x="0" y="0"/>
@@ -2143,4 +3219,701 @@
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="4294967293" verticalDpi="0" r:id="rId1"/>
   <drawing r:id="rId2"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{96742155-2610-4DAA-9890-EC6CFFBE1A57}">
+  <dimension ref="A1:M47"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData>
+    <row r="1" spans="1:13" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="B1" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="C1" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="D1" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="F1" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="G1" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="H1" s="3" t="s">
+        <v>1</v>
+      </c>
+      <c r="J1" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="K1" s="3" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="2" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A2" s="1">
+        <v>0.55317129629629636</v>
+      </c>
+      <c r="B2">
+        <v>251.5</v>
+      </c>
+      <c r="C2">
+        <v>34.914000000000001</v>
+      </c>
+      <c r="D2">
+        <v>6.8000000000000005E-2</v>
+      </c>
+      <c r="F2" s="1">
+        <v>0.55314814814814817</v>
+      </c>
+      <c r="G2">
+        <v>251.6</v>
+      </c>
+      <c r="H2">
+        <v>34.682000000000002</v>
+      </c>
+      <c r="J2" t="str">
+        <f t="shared" ref="J2:J21" si="0">IF(TEXT(A2,"HH:MM")&lt;&gt;TEXT(F2,"HH:MM"),"err","")</f>
+        <v/>
+      </c>
+      <c r="K2" s="2">
+        <f>H2-C2</f>
+        <v>-0.23199999999999932</v>
+      </c>
+      <c r="M2" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="3" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A3" s="1">
+        <v>0.5575</v>
+      </c>
+      <c r="B3">
+        <v>251</v>
+      </c>
+      <c r="C3">
+        <v>36.137999999999998</v>
+      </c>
+      <c r="D3">
+        <v>6.4000000000000001E-2</v>
+      </c>
+      <c r="F3" s="1">
+        <v>0.55748842592592596</v>
+      </c>
+      <c r="G3">
+        <v>251.6</v>
+      </c>
+      <c r="H3">
+        <v>36.226999999999997</v>
+      </c>
+      <c r="J3" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="K3" s="2">
+        <f>H3-C3</f>
+        <v>8.8999999999998636E-2</v>
+      </c>
+    </row>
+    <row r="4" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A4" s="1">
+        <v>0.56276620370370367</v>
+      </c>
+      <c r="B4">
+        <v>250.5</v>
+      </c>
+      <c r="C4">
+        <v>29.506</v>
+      </c>
+      <c r="D4">
+        <v>5.2999999999999999E-2</v>
+      </c>
+      <c r="F4" s="1">
+        <v>0.56276620370370367</v>
+      </c>
+      <c r="G4">
+        <v>250.5</v>
+      </c>
+      <c r="H4">
+        <v>29.507999999999999</v>
+      </c>
+      <c r="J4" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="K4" s="2">
+        <f>H4-C4</f>
+        <v>1.9999999999988916E-3</v>
+      </c>
+    </row>
+    <row r="5" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A5" s="1">
+        <v>0.56406250000000002</v>
+      </c>
+      <c r="B5">
+        <v>250.8</v>
+      </c>
+      <c r="C5">
+        <v>35.067999999999998</v>
+      </c>
+      <c r="D5">
+        <v>6.0999999999999999E-2</v>
+      </c>
+      <c r="F5" s="1">
+        <v>0.56399305555555557</v>
+      </c>
+      <c r="G5">
+        <v>250.5</v>
+      </c>
+      <c r="H5">
+        <v>34.295000000000002</v>
+      </c>
+      <c r="J5" t="str">
+        <f>IF(TEXT(A5,"HH:MM")&lt;&gt;TEXT(F5,"HH:MM"),"err","")</f>
+        <v/>
+      </c>
+      <c r="K5" s="2"/>
+    </row>
+    <row r="6" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A6" s="1">
+        <v>0.5658333333333333</v>
+      </c>
+      <c r="B6">
+        <v>250.2</v>
+      </c>
+      <c r="C6">
+        <v>29.300999999999998</v>
+      </c>
+      <c r="D6">
+        <v>5.0999999999999997E-2</v>
+      </c>
+      <c r="F6" s="1">
+        <v>0.5658333333333333</v>
+      </c>
+      <c r="G6">
+        <v>250.5</v>
+      </c>
+      <c r="H6">
+        <v>29.334</v>
+      </c>
+      <c r="J6" t="str">
+        <f t="shared" ref="J6:J21" si="1">IF(TEXT(A6,"HH:MM")&lt;&gt;TEXT(F6,"HH:MM"),"err","")</f>
+        <v/>
+      </c>
+      <c r="K6" s="2"/>
+    </row>
+    <row r="7" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A7" s="1">
+        <v>0.5669791666666667</v>
+      </c>
+      <c r="B7">
+        <v>250.8</v>
+      </c>
+      <c r="C7">
+        <v>35.588999999999999</v>
+      </c>
+      <c r="D7">
+        <v>6.3E-2</v>
+      </c>
+      <c r="F7" s="1">
+        <v>0.5669791666666667</v>
+      </c>
+      <c r="G7">
+        <v>250.6</v>
+      </c>
+      <c r="H7">
+        <v>35.558999999999997</v>
+      </c>
+      <c r="J7" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+      <c r="K7" s="2">
+        <f t="shared" ref="K7:K21" si="2">H7-C7</f>
+        <v>-3.0000000000001137E-2</v>
+      </c>
+    </row>
+    <row r="8" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A8" s="1">
+        <v>0.57101851851851848</v>
+      </c>
+      <c r="B8">
+        <v>250.4</v>
+      </c>
+      <c r="C8">
+        <v>28.795999999999999</v>
+      </c>
+      <c r="D8">
+        <v>5.0999999999999997E-2</v>
+      </c>
+      <c r="F8" s="1">
+        <v>0.57101851851851848</v>
+      </c>
+      <c r="G8">
+        <v>250.5</v>
+      </c>
+      <c r="H8">
+        <v>28.81</v>
+      </c>
+      <c r="J8" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+      <c r="K8" s="2">
+        <f t="shared" si="2"/>
+        <v>1.3999999999999346E-2</v>
+      </c>
+    </row>
+    <row r="9" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A9" s="1">
+        <v>0.5741087962962963</v>
+      </c>
+      <c r="B9">
+        <v>250.4</v>
+      </c>
+      <c r="C9">
+        <v>28.797999999999998</v>
+      </c>
+      <c r="D9">
+        <v>5.7000000000000002E-2</v>
+      </c>
+      <c r="F9" s="1">
+        <v>0.5741087962962963</v>
+      </c>
+      <c r="G9">
+        <v>251.4</v>
+      </c>
+      <c r="H9">
+        <v>28.742999999999999</v>
+      </c>
+      <c r="J9" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+      <c r="K9" s="2">
+        <f t="shared" si="2"/>
+        <v>-5.4999999999999716E-2</v>
+      </c>
+    </row>
+    <row r="10" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A10" s="1">
+        <v>0.57581018518518523</v>
+      </c>
+      <c r="B10">
+        <v>250.7</v>
+      </c>
+      <c r="C10">
+        <v>35.308999999999997</v>
+      </c>
+      <c r="D10">
+        <v>6.8000000000000005E-2</v>
+      </c>
+      <c r="F10" s="1">
+        <v>0.57581018518518523</v>
+      </c>
+      <c r="G10">
+        <v>250.6</v>
+      </c>
+      <c r="H10">
+        <v>35.296999999999997</v>
+      </c>
+      <c r="J10" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+      <c r="K10" s="2">
+        <f t="shared" si="2"/>
+        <v>-1.2000000000000455E-2</v>
+      </c>
+    </row>
+    <row r="11" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A11" s="1">
+        <v>0.57891203703703698</v>
+      </c>
+      <c r="B11">
+        <v>251.1</v>
+      </c>
+      <c r="C11">
+        <v>35.889000000000003</v>
+      </c>
+      <c r="D11">
+        <v>6.9000000000000006E-2</v>
+      </c>
+      <c r="F11" s="1">
+        <v>0.57891203703703698</v>
+      </c>
+      <c r="G11">
+        <v>250.9</v>
+      </c>
+      <c r="H11">
+        <v>35.857999999999997</v>
+      </c>
+      <c r="J11" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+      <c r="K11" s="2">
+        <f t="shared" si="2"/>
+        <v>-3.1000000000005912E-2</v>
+      </c>
+    </row>
+    <row r="12" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A12" s="1">
+        <v>0.58092592592592596</v>
+      </c>
+      <c r="B12">
+        <v>250.8</v>
+      </c>
+      <c r="C12">
+        <v>28.018999999999998</v>
+      </c>
+      <c r="D12">
+        <v>5.8999999999999997E-2</v>
+      </c>
+      <c r="F12" s="1">
+        <v>0.5809375</v>
+      </c>
+      <c r="G12">
+        <v>250.8</v>
+      </c>
+      <c r="H12">
+        <v>28.018999999999998</v>
+      </c>
+      <c r="J12" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+      <c r="K12" s="2">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A13" s="1">
+        <v>0.58776620370370369</v>
+      </c>
+      <c r="B13">
+        <v>250.2</v>
+      </c>
+      <c r="C13">
+        <v>28.951000000000001</v>
+      </c>
+      <c r="D13">
+        <v>0.06</v>
+      </c>
+      <c r="F13" s="1">
+        <v>0.58776620370370369</v>
+      </c>
+      <c r="G13">
+        <v>250.4</v>
+      </c>
+      <c r="H13">
+        <v>28.969000000000001</v>
+      </c>
+      <c r="J13" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+      <c r="K13" s="2">
+        <f t="shared" si="2"/>
+        <v>1.8000000000000682E-2</v>
+      </c>
+    </row>
+    <row r="14" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A14" s="1">
+        <v>0.58880787037037041</v>
+      </c>
+      <c r="B14">
+        <v>251</v>
+      </c>
+      <c r="C14">
+        <v>35.619999999999997</v>
+      </c>
+      <c r="D14">
+        <v>7.1999999999999995E-2</v>
+      </c>
+      <c r="F14" s="1">
+        <v>0.58878472222222222</v>
+      </c>
+      <c r="G14">
+        <v>250.1</v>
+      </c>
+      <c r="H14">
+        <v>35.479999999999997</v>
+      </c>
+      <c r="J14" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+      <c r="K14" s="2">
+        <f t="shared" si="2"/>
+        <v>-0.14000000000000057</v>
+      </c>
+    </row>
+    <row r="15" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A15" s="1">
+        <v>0.59070601851851856</v>
+      </c>
+      <c r="B15">
+        <v>250.5</v>
+      </c>
+      <c r="C15">
+        <v>28.478000000000002</v>
+      </c>
+      <c r="D15">
+        <v>6.3E-2</v>
+      </c>
+      <c r="F15" s="1">
+        <v>0.59070601851851856</v>
+      </c>
+      <c r="G15">
+        <v>250.9</v>
+      </c>
+      <c r="H15">
+        <v>28.518000000000001</v>
+      </c>
+      <c r="J15" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+      <c r="K15" s="2">
+        <f t="shared" si="2"/>
+        <v>3.9999999999999147E-2</v>
+      </c>
+    </row>
+    <row r="16" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A16" s="1">
+        <v>0.59214120370370371</v>
+      </c>
+      <c r="B16">
+        <v>251.6</v>
+      </c>
+      <c r="C16">
+        <v>34.435000000000002</v>
+      </c>
+      <c r="D16">
+        <v>6.7000000000000004E-2</v>
+      </c>
+      <c r="F16" s="1">
+        <v>0.59214120370370371</v>
+      </c>
+      <c r="G16">
+        <v>250.1</v>
+      </c>
+      <c r="H16">
+        <v>34.478999999999999</v>
+      </c>
+      <c r="J16" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+      <c r="K16" s="2">
+        <f t="shared" si="2"/>
+        <v>4.399999999999693E-2</v>
+      </c>
+    </row>
+    <row r="17" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A17" s="1">
+        <v>0.59946759259259264</v>
+      </c>
+      <c r="B17">
+        <v>251.6</v>
+      </c>
+      <c r="C17">
+        <v>33.265000000000001</v>
+      </c>
+      <c r="D17">
+        <v>5.8999999999999997E-2</v>
+      </c>
+      <c r="F17" s="1">
+        <v>0.59946759259259264</v>
+      </c>
+      <c r="G17">
+        <v>250.5</v>
+      </c>
+      <c r="H17">
+        <v>33.347000000000001</v>
+      </c>
+      <c r="J17" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+      <c r="K17" s="2">
+        <f t="shared" si="2"/>
+        <v>8.2000000000000739E-2</v>
+      </c>
+    </row>
+    <row r="18" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A18" s="1"/>
+      <c r="F18" s="1"/>
+      <c r="J18" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+      <c r="K18" s="2"/>
+    </row>
+    <row r="19" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A19" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="F19" s="1"/>
+      <c r="K19" s="2"/>
+    </row>
+    <row r="20" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A20" s="1"/>
+      <c r="F20" s="1"/>
+      <c r="J20" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+      <c r="K20" s="2"/>
+    </row>
+    <row r="21" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A21" s="1"/>
+      <c r="F21" s="1"/>
+      <c r="J21" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+      <c r="K21" s="2"/>
+    </row>
+    <row r="22" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="K22" s="2"/>
+    </row>
+    <row r="23" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="I23" t="s">
+        <v>4</v>
+      </c>
+      <c r="K23" s="2">
+        <f>MIN($K$2:$K$21)</f>
+        <v>-0.23199999999999932</v>
+      </c>
+    </row>
+    <row r="24" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="I24" t="s">
+        <v>5</v>
+      </c>
+      <c r="K24" s="2">
+        <f>AVERAGE($K$2:$K$21)</f>
+        <v>-1.5071428571429481E-2</v>
+      </c>
+    </row>
+    <row r="25" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="I25" t="s">
+        <v>6</v>
+      </c>
+      <c r="K25" s="2">
+        <f>MAX($K$2:$K$21)</f>
+        <v>8.8999999999998636E-2</v>
+      </c>
+    </row>
+    <row r="26" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="K26" s="2"/>
+    </row>
+    <row r="27" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="F27" s="1"/>
+    </row>
+    <row r="28" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A28" s="1"/>
+      <c r="F28" s="1"/>
+    </row>
+    <row r="29" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A29" s="1"/>
+      <c r="F29" s="1"/>
+    </row>
+    <row r="30" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A30" s="1"/>
+      <c r="F30" s="1"/>
+    </row>
+    <row r="31" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A31" s="1"/>
+      <c r="F31" s="1"/>
+    </row>
+    <row r="32" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A32" s="1"/>
+      <c r="F32" s="1"/>
+    </row>
+    <row r="33" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A33" s="1"/>
+      <c r="F33" s="1"/>
+    </row>
+    <row r="34" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A34" s="1"/>
+      <c r="F34" s="1"/>
+    </row>
+    <row r="35" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A35" s="1"/>
+      <c r="F35" s="1"/>
+    </row>
+    <row r="36" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A36" s="1"/>
+      <c r="F36" s="1"/>
+    </row>
+    <row r="37" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A37" s="1"/>
+      <c r="F37" s="1"/>
+    </row>
+    <row r="38" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A38" s="1"/>
+      <c r="F38" s="1"/>
+    </row>
+    <row r="39" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A39" s="1"/>
+      <c r="F39" s="1"/>
+    </row>
+    <row r="40" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A40" s="1"/>
+      <c r="F40" s="1"/>
+    </row>
+    <row r="41" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A41" s="1"/>
+      <c r="F41" s="1"/>
+    </row>
+    <row r="42" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A42" s="1"/>
+      <c r="F42" s="1"/>
+    </row>
+    <row r="43" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A43" s="1"/>
+      <c r="F43" s="1"/>
+    </row>
+    <row r="44" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A44" s="1"/>
+      <c r="F44" s="1"/>
+    </row>
+    <row r="45" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A45" s="1"/>
+      <c r="F45" s="1"/>
+    </row>
+    <row r="46" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A46" s="1"/>
+      <c r="F46" s="1"/>
+    </row>
+    <row r="47" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A47" s="1"/>
+      <c r="F47" s="1"/>
+    </row>
+  </sheetData>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="F27:H46">
+    <sortCondition ref="F27:F46"/>
+  </sortState>
+  <conditionalFormatting sqref="K2:K17">
+    <cfRule type="colorScale" priority="1">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="max"/>
+        <color theme="7" tint="0.79998168889431442"/>
+        <color rgb="FFFF0000"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="4294967293" verticalDpi="0" r:id="rId1"/>
+  <drawing r:id="rId2"/>
+</worksheet>
 </file>
</xml_diff>